<commit_message>
Update course plans and related documents for various subjects at Dalarna University
- Updated scrape_hash values for course plans GEG26J, GEG2ZQ, GEG2ZR, GSQ25J, GSQ25K, GSQ33N, GMI23G, GMI2J3.
- Corrected typos in course descriptions and assessment sections across multiple course plans.
- Added missing course SS3009 to the list of inactive course plans and updated the count of courses in the Swedish as a Second Language MOC.
- Updated binary files related to analysis and examination forms for IHV, IKS, and ISLL departments.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Samstämmighet svenska och engelska.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Samstämmighet svenska och engelska.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Samstämmighet svenska och engel" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Samstämmighet svenska och engel'!$A$1:$E$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Samstämmighet svenska och engel'!$A$1:$E$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -472,12 +472,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>IK1064</t>
+          <t>AMD238</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -487,19 +487,19 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Svenska: 12 mål, engelska: 0 mål (diff 12)</t>
+          <t>Svenska: 17 mål, engelska: 0 mål (diff 17)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1064</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMD238</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>AMD238</t>
+          <t>AMD239</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -519,14 +519,14 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMD238</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMD239</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>AMD239</t>
+          <t>GMD2AR</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -541,19 +541,19 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Svenska: 17 mål, engelska: 0 mål (diff 17)</t>
+          <t>Svenska: 28 mål, engelska: 0 mål (diff 28)</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMD239</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2AR</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>GMD2AR</t>
+          <t>GMD2GF</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -568,19 +568,19 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Svenska: 28 mål, engelska: 0 mål (diff 28)</t>
+          <t>Svenska: 24 mål, engelska: 1 mål (diff 23)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2AR</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2GF</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>GMD2GF</t>
+          <t>GMD2GG</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -600,14 +600,14 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2GF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2GG</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>GMD2GG</t>
+          <t>GMD2H3</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -622,19 +622,19 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Svenska: 24 mål, engelska: 1 mål (diff 23)</t>
+          <t>Svenska: 8 mål, engelska: 0 mål (diff 8)</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2GG</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H3</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>GMD2H3</t>
+          <t>GMD2MH</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -649,19 +649,19 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Svenska: 8 mål, engelska: 0 mål (diff 8)</t>
+          <t>Svenska: 10 mål, engelska: 0 mål (diff 10)</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H3</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2MH</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>GMD2MH</t>
+          <t>GMD2TV</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -676,19 +676,19 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Svenska: 10 mål, engelska: 0 mål (diff 10)</t>
+          <t>Svenska: 32 mål, engelska: 0 mål (diff 32)</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2MH</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2TV</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>GMD2TV</t>
+          <t>GMD2XQ</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -703,19 +703,19 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Svenska: 32 mål, engelska: 0 mål (diff 32)</t>
+          <t>Svenska: 77 mål, engelska: 0 mål (diff 77)</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2TV</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2XQ</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>GMD2XQ</t>
+          <t>GMD33X</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -730,19 +730,19 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Svenska: 77 mål, engelska: 0 mål (diff 77)</t>
+          <t>Svenska: 45 mål, engelska: 0 mål (diff 45)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2XQ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD33X</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>GMD33X</t>
+          <t>GMD33Y</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -757,24 +757,24 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Svenska: 45 mål, engelska: 0 mål (diff 45)</t>
+          <t>Svenska: 77 mål, engelska: 0 mål (diff 77)</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD33X</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD33Y</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>GMD33Y</t>
+          <t>MT1033</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -784,19 +784,19 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Svenska: 77 mål, engelska: 0 mål (diff 77)</t>
+          <t>Svenska: 1 mål, engelska: 0 mål (diff 1)</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD33Y</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1033</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>MT1033</t>
+          <t>MT1060</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -811,19 +811,19 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Svenska: 1 mål, engelska: 0 mål (diff 1)</t>
+          <t>Svenska: 10 mål, engelska: 9 mål (diff 1)</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1033</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1060</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>MT1060</t>
+          <t>MT2006</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -838,24 +838,24 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Svenska: 10 mål, engelska: 9 mål (diff 1)</t>
+          <t>Svenska: 3 mål, engelska: 0 mål (diff 3)</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1060</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT2006</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>MT2006</t>
+          <t>GSQ23K</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -865,24 +865,24 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Svenska: 3 mål, engelska: 0 mål (diff 3)</t>
+          <t>Svenska: 5 mål, engelska: 4 mål (diff 1)</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT2006</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23K</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>GSQ23K</t>
+          <t>ST1013</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>STA</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -892,44 +892,17 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Svenska: 5 mål, engelska: 4 mål (diff 1)</t>
+          <t>Svenska: 8 mål, engelska: 0 mål (diff 8)</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23K</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>ST1013</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>STA</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Paritetsskillnad</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Svenska: 8 mål, engelska: 0 mål (diff 8)</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ST1013</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E18"/>
+  <autoFilter ref="A1:E17"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
@@ -963,8 +936,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId30"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A17" r:id="rId31"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A18" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId34"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update analysis spreadsheets for consistency and accuracy in Swedish and English language usage
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Samstämmighet svenska och engelska.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Samstämmighet svenska och engelska.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Samstämmighet svenska och engel" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Samstämmighet svenska och engel'!$A$1:$E$130</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Samstämmighet svenska och engel'!$A$1:$E$142</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E130"/>
+  <dimension ref="A1:E142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2173,7 +2173,7 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>AMD239</t>
+          <t>AMD238</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2183,24 +2183,24 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Paritetsskillnad</t>
+          <t>Saknar punktlista (en)</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Svenska: 17 mål, engelska: 2 mål (diff 15)</t>
+          <t>Learning Outcomes skrivet som löpande text (2 mål utan punktlista)</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMD239</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMD238</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>GMD2AR</t>
+          <t>AMD239</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2215,19 +2215,19 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Svenska: 28 mål, engelska: 1 mål (diff 27)</t>
+          <t>Svenska: 17 mål, engelska: 2 mål (diff 15)</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2AR</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMD239</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>GMD2BH</t>
+          <t>AMD239</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2237,24 +2237,24 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Paritetsskillnad</t>
+          <t>Saknar punktlista (en)</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Svenska: 6 mål, engelska: 0 mål (diff 6)</t>
+          <t>Learning Outcomes skrivet som löpande text (2 mål utan punktlista)</t>
         </is>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2BH</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMD239</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>GMD2EX</t>
+          <t>GMD2AR</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2269,19 +2269,19 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Svenska: 8 mål, engelska: 0 mål (diff 8)</t>
+          <t>Svenska: 28 mål, engelska: 1 mål (diff 27)</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2EX</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2AR</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>GMD2GF</t>
+          <t>GMD2AR</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2291,24 +2291,24 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Paritetsskillnad</t>
+          <t>Saknar punktlista (en)</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Svenska: 24 mål, engelska: 1 mål (diff 23)</t>
+          <t>Learning Outcomes skrivet som löpande text (1 mål utan punktlista)</t>
         </is>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2GF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2AR</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>GMD2GG</t>
+          <t>GMD2BH</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2323,19 +2323,19 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Svenska: 24 mål, engelska: 1 mål (diff 23)</t>
+          <t>Svenska: 6 mål, engelska: 0 mål (diff 6)</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2GG</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2BH</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>GMD2GU</t>
+          <t>GMD2EX</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2350,19 +2350,19 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Svenska: 5 mål, engelska: 0 mål (diff 5)</t>
+          <t>Svenska: 8 mål, engelska: 0 mål (diff 8)</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2GU</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2EX</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>GMD2H5</t>
+          <t>GMD2GF</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2377,19 +2377,19 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Svenska: 8 mål, engelska: 0 mål (diff 8)</t>
+          <t>Svenska: 24 mål, engelska: 1 mål (diff 23)</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2GF</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>GMD2HE</t>
+          <t>GMD2GG</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2404,19 +2404,19 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Svenska: 7 mål, engelska: 0 mål (diff 7)</t>
+          <t>Svenska: 24 mål, engelska: 1 mål (diff 23)</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HE</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2GG</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>GMD2HF</t>
+          <t>GMD2GU</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2431,19 +2431,19 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Svenska: 7 mål, engelska: 0 mål (diff 7)</t>
+          <t>Svenska: 5 mål, engelska: 0 mål (diff 5)</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2GU</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>GMD2HG</t>
+          <t>GMD2H3</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2453,24 +2453,24 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Paritetsskillnad</t>
+          <t>Saknar punktlista (en)</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Svenska: 9 mål, engelska: 0 mål (diff 9)</t>
+          <t>Learning Outcomes skrivet som löpande text (8 mål utan punktlista)</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HG</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H3</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>GMD2HH</t>
+          <t>GMD2H5</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2485,19 +2485,19 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Svenska: 7 mål, engelska: 0 mål (diff 7)</t>
+          <t>Svenska: 8 mål, engelska: 0 mål (diff 8)</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HH</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H5</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>GMD2HJ</t>
+          <t>GMD2HE</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2517,14 +2517,14 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HJ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HE</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>GMD2HK</t>
+          <t>GMD2HF</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2539,19 +2539,19 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Svenska: 9 mål, engelska: 0 mål (diff 9)</t>
+          <t>Svenska: 7 mål, engelska: 0 mål (diff 7)</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HK</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HF</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>GMD2MH</t>
+          <t>GMD2HG</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2566,19 +2566,19 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Svenska: 10 mål, engelska: 8 mål (diff 2)</t>
+          <t>Svenska: 9 mål, engelska: 0 mål (diff 9)</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2MH</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HG</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>GMD2MJ</t>
+          <t>GMD2HH</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2593,19 +2593,19 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Svenska: 10 mål, engelska: 0 mål (diff 10)</t>
+          <t>Svenska: 7 mål, engelska: 0 mål (diff 7)</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2MJ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HH</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>GMD2PA</t>
+          <t>GMD2HJ</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2620,19 +2620,19 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Svenska: 6 mål, engelska: 0 mål (diff 6)</t>
+          <t>Svenska: 7 mål, engelska: 0 mål (diff 7)</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2PA</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HJ</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>GMD2TV</t>
+          <t>GMD2HK</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2647,19 +2647,19 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Svenska: 32 mål, engelska: 2 mål (diff 30)</t>
+          <t>Svenska: 9 mål, engelska: 0 mål (diff 9)</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2TV</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HK</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>GMD2XQ</t>
+          <t>GMD2MH</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2674,19 +2674,19 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Svenska: 77 mål, engelska: 2 mål (diff 75)</t>
+          <t>Svenska: 10 mål, engelska: 8 mål (diff 2)</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2XQ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2MH</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>GMD33X</t>
+          <t>GMD2MH</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2696,24 +2696,24 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Paritetsskillnad</t>
+          <t>Saknar punktlista (en)</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Svenska: 45 mål, engelska: 7 mål (diff 38)</t>
+          <t>Learning Outcomes skrivet som löpande text (8 mål utan punktlista)</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD33X</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2MH</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>GMD33Y</t>
+          <t>GMD2MJ</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2728,19 +2728,19 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Svenska: 77 mål, engelska: 2 mål (diff 75)</t>
+          <t>Svenska: 10 mål, engelska: 0 mål (diff 10)</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD33Y</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2MJ</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>GMD3FX</t>
+          <t>GMD2PA</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2755,19 +2755,19 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Svenska: 4 mål, engelska: 0 mål (diff 4)</t>
+          <t>Svenska: 6 mål, engelska: 0 mål (diff 6)</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD3FX</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2PA</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>GMD3GZ</t>
+          <t>GMD2TV</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2782,19 +2782,19 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Svenska: 6 mål, engelska: 0 mål (diff 6)</t>
+          <t>Svenska: 32 mål, engelska: 2 mål (diff 30)</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD3GZ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2TV</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>MD1085</t>
+          <t>GMD2TV</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2804,24 +2804,24 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Paritetsskillnad</t>
+          <t>Saknar punktlista (en)</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Svenska: 5 mål, engelska: 0 mål (diff 5)</t>
+          <t>Learning Outcomes skrivet som löpande text (2 mål utan punktlista)</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1085</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2TV</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>MD1103</t>
+          <t>GMD2XQ</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2836,19 +2836,19 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Svenska: 6 mål, engelska: 0 mål (diff 6)</t>
+          <t>Svenska: 77 mål, engelska: 2 mål (diff 75)</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1103</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2XQ</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>MD2022</t>
+          <t>GMD2XQ</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2858,24 +2858,24 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Paritetsskillnad</t>
+          <t>Saknar punktlista (en)</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Svenska: 17 mål, engelska: 0 mål (diff 17)</t>
+          <t>Learning Outcomes skrivet som löpande text (2 mål utan punktlista)</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD2022</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2XQ</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>MD2023</t>
+          <t>GMD33X</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2890,19 +2890,19 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Svenska: 2 mål, engelska: 0 mål (diff 2)</t>
+          <t>Svenska: 45 mål, engelska: 7 mål (diff 38)</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD2023</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD33X</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>MD2024</t>
+          <t>GMD33X</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2912,24 +2912,24 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Paritetsskillnad</t>
+          <t>Saknar punktlista (en)</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Svenska: 3 mål, engelska: 0 mål (diff 3)</t>
+          <t>Learning Outcomes skrivet som löpande text (7 mål utan punktlista)</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD2024</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD33X</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>MD2025</t>
+          <t>GMD33Y</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2944,19 +2944,19 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Svenska: 6 mål, engelska: 0 mål (diff 6)</t>
+          <t>Svenska: 77 mål, engelska: 2 mål (diff 75)</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD2025</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD33Y</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>MD2026</t>
+          <t>GMD33Y</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2966,29 +2966,29 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Paritetsskillnad</t>
+          <t>Saknar punktlista (en)</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Svenska: 6 mål, engelska: 0 mål (diff 6)</t>
+          <t>Learning Outcomes skrivet som löpande text (2 mål utan punktlista)</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD2026</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD33Y</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>GMT2WL</t>
+          <t>GMD3FX</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -3003,19 +3003,19 @@
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT2WL</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD3FX</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>GMT34A</t>
+          <t>GMD3GZ</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -3025,24 +3025,24 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Svenska: 8 mål, engelska: 0 mål (diff 8)</t>
+          <t>Svenska: 6 mål, engelska: 0 mål (diff 6)</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT34A</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD3GZ</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>GMT34K</t>
+          <t>MD1085</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -3057,19 +3057,19 @@
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT34K</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1085</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>GMT34L</t>
+          <t>MD1103</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -3079,24 +3079,24 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Svenska: 5 mål, engelska: 0 mål (diff 5)</t>
+          <t>Svenska: 6 mål, engelska: 0 mål (diff 6)</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT34L</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD1103</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>GMT34P</t>
+          <t>MD2022</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -3106,24 +3106,24 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Svenska: 5 mål, engelska: 0 mål (diff 5)</t>
+          <t>Svenska: 17 mål, engelska: 0 mål (diff 17)</t>
         </is>
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT34P</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD2022</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>GMT34W</t>
+          <t>MD2023</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -3133,24 +3133,24 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Svenska: 6 mål, engelska: 0 mål (diff 6)</t>
+          <t>Svenska: 2 mål, engelska: 0 mål (diff 2)</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT34W</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD2023</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>GMT3BW</t>
+          <t>MD2024</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -3160,24 +3160,24 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Svenska: 7 mål, engelska: 0 mål (diff 7)</t>
+          <t>Svenska: 3 mål, engelska: 0 mål (diff 3)</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3BW</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD2024</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>GMT3JZ</t>
+          <t>MD2025</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -3187,24 +3187,24 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Svenska: 4 mål, engelska: 0 mål (diff 4)</t>
+          <t>Svenska: 6 mål, engelska: 0 mål (diff 6)</t>
         </is>
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JZ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD2025</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>MT1060</t>
+          <t>MD2026</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -3214,19 +3214,19 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Svenska: 10 mål, engelska: 9 mål (diff 1)</t>
+          <t>Svenska: 6 mål, engelska: 0 mål (diff 6)</t>
         </is>
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1060</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MD2026</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>MT1068</t>
+          <t>GMT2WL</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -3241,19 +3241,19 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Svenska: 6 mål, engelska: 0 mål (diff 6)</t>
+          <t>Svenska: 4 mål, engelska: 0 mål (diff 4)</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1068</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT2WL</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>MT1074</t>
+          <t>GMT34A</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -3268,19 +3268,19 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Svenska: 3 mål, engelska: 0 mål (diff 3)</t>
+          <t>Svenska: 8 mål, engelska: 0 mål (diff 8)</t>
         </is>
       </c>
       <c r="E105" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1074</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT34A</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>MT2006</t>
+          <t>GMT34K</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -3295,24 +3295,24 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Svenska: 3 mål, engelska: 1 mål (diff 2)</t>
+          <t>Svenska: 5 mål, engelska: 0 mål (diff 5)</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT2006</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT34K</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>BEG222</t>
+          <t>GMT34L</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -3322,24 +3322,24 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Svenska: 4 mål, engelska: 0 mål (diff 4)</t>
+          <t>Svenska: 5 mål, engelska: 0 mål (diff 5)</t>
         </is>
       </c>
       <c r="E107" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BEG222</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT34L</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>GEG2JP</t>
+          <t>GMT34P</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -3349,24 +3349,24 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Svenska: 8 mål, engelska: 0 mål (diff 8)</t>
+          <t>Svenska: 5 mål, engelska: 0 mål (diff 5)</t>
         </is>
       </c>
       <c r="E108" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2JP</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT34P</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>GEG2UE</t>
+          <t>GMT34W</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -3376,24 +3376,24 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Svenska: 7 mål, engelska: 0 mål (diff 7)</t>
+          <t>Svenska: 6 mål, engelska: 0 mål (diff 6)</t>
         </is>
       </c>
       <c r="E109" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2UE</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT34W</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>GEG2ZQ</t>
+          <t>GMT3BW</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -3403,24 +3403,24 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Svenska: 4 mål, engelska: 0 mål (diff 4)</t>
+          <t>Svenska: 7 mål, engelska: 0 mål (diff 7)</t>
         </is>
       </c>
       <c r="E110" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2ZQ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3BW</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>GEG33B</t>
+          <t>GMT3JZ</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -3430,51 +3430,51 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Svenska: 6 mål, engelska: 0 mål (diff 6)</t>
+          <t>Svenska: 4 mål, engelska: 0 mål (diff 4)</t>
         </is>
       </c>
       <c r="E111" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG33B</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JZ</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>GEG38F</t>
+          <t>MT1033</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Paritetsskillnad</t>
+          <t>Saknar punktlista (en)</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Svenska: 3 mål, engelska: 0 mål (diff 3)</t>
+          <t>Learning Outcomes skrivet som löpande text (1 mål utan punktlista)</t>
         </is>
       </c>
       <c r="E112" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG38F</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1033</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>GSQ23J</t>
+          <t>MT1060</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -3484,24 +3484,24 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Svenska: 8 mål, engelska: 0 mål (diff 8)</t>
+          <t>Svenska: 10 mål, engelska: 9 mål (diff 1)</t>
         </is>
       </c>
       <c r="E113" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23J</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1060</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>GSQ23K</t>
+          <t>MT1068</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -3511,24 +3511,24 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Svenska: 5 mål, engelska: 4 mål (diff 1)</t>
+          <t>Svenska: 6 mål, engelska: 0 mål (diff 6)</t>
         </is>
       </c>
       <c r="E114" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23K</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1068</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>GSQ25J</t>
+          <t>MT1074</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -3538,24 +3538,24 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Svenska: 6 mål, engelska: 0 mål (diff 6)</t>
+          <t>Svenska: 3 mål, engelska: 0 mål (diff 3)</t>
         </is>
       </c>
       <c r="E115" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25J</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1074</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>GSQ25N</t>
+          <t>MT2006</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -3565,51 +3565,51 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Svenska: 10 mål, engelska: 0 mål (diff 10)</t>
+          <t>Svenska: 3 mål, engelska: 1 mål (diff 2)</t>
         </is>
       </c>
       <c r="E116" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25N</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT2006</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>GSQ2DH</t>
+          <t>MT2006</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Paritetsskillnad</t>
+          <t>Saknar punktlista (en)</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Svenska: 5 mål, engelska: 0 mål (diff 5)</t>
+          <t>Learning Outcomes skrivet som löpande text (1 mål utan punktlista)</t>
         </is>
       </c>
       <c r="E117" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2DH</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT2006</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>GSQ2H7</t>
+          <t>BEG222</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -3619,24 +3619,24 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Svenska: 6 mål, engelska: 0 mål (diff 6)</t>
+          <t>Svenska: 4 mål, engelska: 0 mål (diff 4)</t>
         </is>
       </c>
       <c r="E118" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2H7</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BEG222</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>GSQ2L9</t>
+          <t>GEG2JP</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -3646,24 +3646,24 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Svenska: 4 mål, engelska: 0 mål (diff 4)</t>
+          <t>Svenska: 8 mål, engelska: 0 mål (diff 8)</t>
         </is>
       </c>
       <c r="E119" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2L9</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2JP</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>GSQ2MC</t>
+          <t>GEG2UE</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -3673,24 +3673,24 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Svenska: 6 mål, engelska: 0 mål (diff 6)</t>
+          <t>Svenska: 7 mål, engelska: 0 mål (diff 7)</t>
         </is>
       </c>
       <c r="E120" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2MC</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2UE</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>GSQ2PH</t>
+          <t>GEG2ZQ</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -3700,24 +3700,24 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Svenska: 6 mål, engelska: 0 mål (diff 6)</t>
+          <t>Svenska: 4 mål, engelska: 0 mål (diff 4)</t>
         </is>
       </c>
       <c r="E121" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2PH</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2ZQ</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>GSQ2R5</t>
+          <t>GEG33B</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -3727,24 +3727,24 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Svenska: 5 mål, engelska: 0 mål (diff 5)</t>
+          <t>Svenska: 6 mål, engelska: 0 mål (diff 6)</t>
         </is>
       </c>
       <c r="E122" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2R5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG33B</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>GSQ2VY</t>
+          <t>GEG38F</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -3754,19 +3754,19 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Svenska: 5 mål, engelska: 0 mål (diff 5)</t>
+          <t>Svenska: 3 mål, engelska: 0 mål (diff 3)</t>
         </is>
       </c>
       <c r="E123" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2VY</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG38F</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>GSQ2WM</t>
+          <t>GSQ23J</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3781,19 +3781,19 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Svenska: 4 mål, engelska: 0 mål (diff 4)</t>
+          <t>Svenska: 8 mål, engelska: 0 mål (diff 8)</t>
         </is>
       </c>
       <c r="E124" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2WM</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23J</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>GSQ2Y2</t>
+          <t>GSQ23K</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3808,19 +3808,19 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Svenska: 6 mål, engelska: 0 mål (diff 6)</t>
+          <t>Svenska: 5 mål, engelska: 4 mål (diff 1)</t>
         </is>
       </c>
       <c r="E125" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2Y2</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23K</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>SQ1003</t>
+          <t>GSQ25J</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3840,19 +3840,19 @@
       </c>
       <c r="E126" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SQ1003</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25J</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>GST2CL</t>
+          <t>GSQ25N</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>STA</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -3862,24 +3862,24 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Svenska: 7 mål, engelska: 0 mål (diff 7)</t>
+          <t>Svenska: 10 mål, engelska: 0 mål (diff 10)</t>
         </is>
       </c>
       <c r="E127" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GST2CL</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25N</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>ST1013</t>
+          <t>GSQ2DH</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>STA</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -3889,24 +3889,24 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Svenska: 8 mål, engelska: 1 mål (diff 7)</t>
+          <t>Svenska: 5 mål, engelska: 0 mål (diff 5)</t>
         </is>
       </c>
       <c r="E128" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ST1013</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2DH</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>GMI24H</t>
+          <t>GSQ2H7</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>XYZ</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -3916,44 +3916,368 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Svenska: 5 mål, engelska: 0 mål (diff 5)</t>
+          <t>Svenska: 6 mål, engelska: 0 mål (diff 6)</t>
         </is>
       </c>
       <c r="E129" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI24H</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2H7</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
+          <t>GSQ2L9</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>SQQ</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Paritetsskillnad</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Svenska: 4 mål, engelska: 0 mål (diff 4)</t>
+        </is>
+      </c>
+      <c r="E130" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2L9</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>GSQ2MC</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>SQQ</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Paritetsskillnad</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Svenska: 6 mål, engelska: 0 mål (diff 6)</t>
+        </is>
+      </c>
+      <c r="E131" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2MC</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>GSQ2PH</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>SQQ</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Paritetsskillnad</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>Svenska: 6 mål, engelska: 0 mål (diff 6)</t>
+        </is>
+      </c>
+      <c r="E132" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2PH</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="inlineStr">
+        <is>
+          <t>GSQ2R5</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>SQQ</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Paritetsskillnad</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Svenska: 5 mål, engelska: 0 mål (diff 5)</t>
+        </is>
+      </c>
+      <c r="E133" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2R5</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>GSQ2VY</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>SQQ</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Paritetsskillnad</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Svenska: 5 mål, engelska: 0 mål (diff 5)</t>
+        </is>
+      </c>
+      <c r="E134" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2VY</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="inlineStr">
+        <is>
+          <t>GSQ2WM</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>SQQ</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Paritetsskillnad</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Svenska: 4 mål, engelska: 0 mål (diff 4)</t>
+        </is>
+      </c>
+      <c r="E135" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2WM</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>GSQ2Y2</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>SQQ</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Paritetsskillnad</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Svenska: 6 mål, engelska: 0 mål (diff 6)</t>
+        </is>
+      </c>
+      <c r="E136" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ2Y2</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="inlineStr">
+        <is>
+          <t>SQ1003</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>SQQ</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Paritetsskillnad</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Svenska: 6 mål, engelska: 0 mål (diff 6)</t>
+        </is>
+      </c>
+      <c r="E137" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=SQ1003</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>GST2CL</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>STA</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Paritetsskillnad</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Svenska: 7 mål, engelska: 0 mål (diff 7)</t>
+        </is>
+      </c>
+      <c r="E138" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GST2CL</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="inlineStr">
+        <is>
+          <t>ST1013</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>STA</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Paritetsskillnad</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Svenska: 8 mål, engelska: 1 mål (diff 7)</t>
+        </is>
+      </c>
+      <c r="E139" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ST1013</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>ST1013</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>STA</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Saknar punktlista (en)</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Learning Outcomes skrivet som löpande text (1 mål utan punktlista)</t>
+        </is>
+      </c>
+      <c r="E140" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ST1013</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>GMI24H</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>XYZ</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Paritetsskillnad</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Svenska: 5 mål, engelska: 0 mål (diff 5)</t>
+        </is>
+      </c>
+      <c r="E141" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI24H</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
           <t>GMI2C8</t>
         </is>
       </c>
-      <c r="B130" t="inlineStr">
+      <c r="B142" t="inlineStr">
         <is>
           <t>XYZ</t>
         </is>
       </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t>Paritetsskillnad</t>
-        </is>
-      </c>
-      <c r="D130" t="inlineStr">
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Paritetsskillnad</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
         <is>
           <t>Svenska: 9 mål, engelska: 0 mål (diff 9)</t>
         </is>
       </c>
-      <c r="E130" s="2" t="inlineStr">
+      <c r="E142" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI2C8</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E130"/>
+  <autoFilter ref="A1:E142"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
@@ -4213,6 +4537,30 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E129" r:id="rId256"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A130" r:id="rId257"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E130" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A131" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E131" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A132" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E132" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A133" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E133" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A134" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E134" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A135" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E135" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A136" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E136" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A137" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E137" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A138" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E138" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A139" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E139" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A140" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E140" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A141" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E141" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A142" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E142" r:id="rId282"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>